<commit_message>
Oct 28 2025 opp changes
</commit_message>
<xml_diff>
--- a/TestData/LV_T1177_CompaniesAddFROpportunityInCompanyDetailPage.xlsx
+++ b/TestData/LV_T1177_CompaniesAddFROpportunityInCompanyDetailPage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBAB9507-05FF-4E88-AF47-B824DC19370A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D73B5E01-B08B-4F1D-8646-B0B2B16D469B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="3" r:id="rId1"/>
@@ -163,9 +163,6 @@
     <t>FR</t>
   </si>
   <si>
-    <t>Debtor Advisors</t>
-  </si>
-  <si>
     <t>TotalDebt</t>
   </si>
   <si>
@@ -215,6 +212,9 @@
   </si>
   <si>
     <t>BUS - Business Services</t>
+  </si>
+  <si>
+    <t>Company-side Advisory</t>
   </si>
 </sst>
 </file>
@@ -546,30 +546,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B2" t="s">
-        <v>54</v>
-      </c>
       <c r="C2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -580,19 +580,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE0366B9-FC69-4100-8413-28CC5C60CF45}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>55</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -603,19 +603,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6F92D56-45BD-4912-85CE-3B5F15739CCA}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -626,14 +626,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -644,7 +644,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -655,7 +655,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -663,7 +663,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -671,10 +671,10 @@
         <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -682,7 +682,7 @@
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -693,28 +693,28 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AC3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -764,7 +764,7 @@
         <v>27</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="R1" s="1" t="s">
         <v>28</v>
@@ -779,16 +779,16 @@
         <v>31</v>
       </c>
       <c r="AA1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AB1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AC1" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -796,10 +796,10 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="D2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E2" t="s">
         <v>32</v>
@@ -820,16 +820,16 @@
         <v>33</v>
       </c>
       <c r="K2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L2" t="s">
         <v>35</v>
       </c>
       <c r="M2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O2" t="s">
         <v>43</v>
@@ -859,10 +859,10 @@
         <v>38</v>
       </c>
       <c r="AC2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
       <c r="M3" t="s">
         <v>36</v>
       </c>

</xml_diff>